<commit_message>
Extend Boston FAF zone analysis to all 2017-2024 annual estimate years
Reshapes FAF5 data to long format (year, tons, value) filtered to zone
251, then updates totals, top-10 destinations/products, mode share, and
import sections to group by year instead of hardcoding 2017 columns.
Also fixes three pre-existing bugs: undefined top_ten_exports variable,
faf_5_modes typo, and a missing pipe before write_xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/top_ten_imp_val.xlsx
+++ b/data/top_ten_imp_val.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -362,10 +362,15 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>total_value</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -378,9 +383,12 @@
         </is>
       </c>
       <c r="B2">
+        <v>2017</v>
+      </c>
+      <c r="C2">
         <v>22.563254868</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Mixed freight</t>
         </is>
@@ -389,133 +397,1420 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B3">
-        <v>19.82979635</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Electronics</t>
+        <v>2018</v>
+      </c>
+      <c r="C3">
+        <v>22.424935147</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mixed freight</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B4">
-        <v>13.147697112</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Pharmaceuticals</t>
+        <v>2019</v>
+      </c>
+      <c r="C4">
+        <v>22.050052484</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mixed freight</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B5">
-        <v>12.117560532</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Misc. mfg. prods.</t>
+        <v>2021</v>
+      </c>
+      <c r="C5">
+        <v>21.950277688</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Mixed freight</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B6">
-        <v>11.976296982</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Precision instruments</t>
+        <v>2020</v>
+      </c>
+      <c r="C6">
+        <v>21.908817899</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Mixed freight</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B7">
-        <v>11.335657705</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Motorized vehicles</t>
+        <v>2023</v>
+      </c>
+      <c r="C7">
+        <v>21.60464556</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Mixed freight</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B8">
-        <v>9.34841215</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Textiles/leather</t>
+        <v>2024</v>
+      </c>
+      <c r="C8">
+        <v>21.550885787</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Mixed freight</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B9">
-        <v>8.335137311</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Machinery</t>
+        <v>2022</v>
+      </c>
+      <c r="C9">
+        <v>21.453375756</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Mixed freight</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>35</t>
         </is>
       </c>
       <c r="B10">
-        <v>7.933302637</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Plastics/rubber</t>
+        <v>2022</v>
+      </c>
+      <c r="C10">
+        <v>20.664648327</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Electronics</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>2021</v>
+      </c>
+      <c r="C11">
+        <v>20.496012635</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>2023</v>
+      </c>
+      <c r="C12">
+        <v>20.212253286</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>2017</v>
+      </c>
+      <c r="C13">
+        <v>19.82979635</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B14">
+        <v>2024</v>
+      </c>
+      <c r="C14">
+        <v>19.800400492</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B15">
+        <v>2018</v>
+      </c>
+      <c r="C15">
+        <v>19.606980378</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B16">
+        <v>2019</v>
+      </c>
+      <c r="C16">
+        <v>18.91087282</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B17">
+        <v>2020</v>
+      </c>
+      <c r="C17">
+        <v>18.863957827</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B18">
+        <v>2024</v>
+      </c>
+      <c r="C18">
+        <v>15.336451874</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B19">
+        <v>2023</v>
+      </c>
+      <c r="C19">
+        <v>14.240153149</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B20">
+        <v>2022</v>
+      </c>
+      <c r="C20">
+        <v>14.195971537</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B21">
+        <v>2019</v>
+      </c>
+      <c r="C21">
+        <v>13.22208058</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B22">
+        <v>2017</v>
+      </c>
+      <c r="C22">
+        <v>13.147697112</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B23">
+        <v>2021</v>
+      </c>
+      <c r="C23">
+        <v>13.007627208</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Misc. mfg. prods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B24">
+        <v>2020</v>
+      </c>
+      <c r="C24">
+        <v>12.925027427</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Misc. mfg. prods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B25">
+        <v>2021</v>
+      </c>
+      <c r="C25">
+        <v>12.729998436</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B26">
+        <v>2018</v>
+      </c>
+      <c r="C26">
+        <v>12.151812909</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B27">
+        <v>2017</v>
+      </c>
+      <c r="C27">
+        <v>12.117560532</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Misc. mfg. prods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B28">
+        <v>2018</v>
+      </c>
+      <c r="C28">
+        <v>12.053701458</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Precision instruments</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B29">
+        <v>2021</v>
+      </c>
+      <c r="C29">
+        <v>12.02595023</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Precision instruments</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B30">
+        <v>2017</v>
+      </c>
+      <c r="C30">
+        <v>11.976296982</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Precision instruments</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B31">
+        <v>2018</v>
+      </c>
+      <c r="C31">
+        <v>11.804498361</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Misc. mfg. prods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B32">
+        <v>2020</v>
+      </c>
+      <c r="C32">
+        <v>11.76864921</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B33">
+        <v>2018</v>
+      </c>
+      <c r="C33">
+        <v>11.7157602</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Motorized vehicles</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B34">
+        <v>2019</v>
+      </c>
+      <c r="C34">
+        <v>11.708666003</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Precision instruments</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B35">
+        <v>2022</v>
+      </c>
+      <c r="C35">
+        <v>11.688858687</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Misc. mfg. prods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B36">
+        <v>2019</v>
+      </c>
+      <c r="C36">
+        <v>11.56394589</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Misc. mfg. prods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37">
+        <v>2019</v>
+      </c>
+      <c r="C37">
+        <v>11.492383889</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Motorized vehicles</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B38">
+        <v>2024</v>
+      </c>
+      <c r="C38">
+        <v>11.489950168</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Motorized vehicles</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B39">
+        <v>2022</v>
+      </c>
+      <c r="C39">
+        <v>11.440443032</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Precision instruments</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B40">
+        <v>2023</v>
+      </c>
+      <c r="C40">
+        <v>11.405761791</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Motorized vehicles</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B41">
+        <v>2020</v>
+      </c>
+      <c r="C41">
+        <v>11.399923779</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Precision instruments</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B42">
+        <v>2017</v>
+      </c>
+      <c r="C42">
+        <v>11.335657705</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Motorized vehicles</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B43">
+        <v>2022</v>
+      </c>
+      <c r="C43">
+        <v>11.251168751</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Motorized vehicles</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B44">
+        <v>2023</v>
+      </c>
+      <c r="C44">
+        <v>11.015596751</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Precision instruments</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B45">
+        <v>2024</v>
+      </c>
+      <c r="C45">
+        <v>10.99514825</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Precision instruments</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B46">
+        <v>2021</v>
+      </c>
+      <c r="C46">
+        <v>10.666123471</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Motorized vehicles</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B47">
+        <v>2023</v>
+      </c>
+      <c r="C47">
+        <v>10.503970719</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Misc. mfg. prods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B48">
+        <v>2020</v>
+      </c>
+      <c r="C48">
+        <v>10.111668516</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Motorized vehicles</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B49">
+        <v>2024</v>
+      </c>
+      <c r="C49">
+        <v>9.960329438999999</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Misc. mfg. prods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B50">
+        <v>2017</v>
+      </c>
+      <c r="C50">
+        <v>9.34841215</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Textiles/leather</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B51">
+        <v>2018</v>
+      </c>
+      <c r="C51">
+        <v>9.155250655</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Textiles/leather</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B52">
+        <v>2021</v>
+      </c>
+      <c r="C52">
+        <v>9.094969187999999</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B53">
+        <v>2022</v>
+      </c>
+      <c r="C53">
+        <v>9.031668614000001</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B54">
+        <v>2018</v>
+      </c>
+      <c r="C54">
+        <v>9.007596475</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B55">
+        <v>2019</v>
+      </c>
+      <c r="C55">
+        <v>8.944119272</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B56">
+        <v>2019</v>
+      </c>
+      <c r="C56">
+        <v>8.799151495</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Textiles/leather</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B57">
+        <v>2024</v>
+      </c>
+      <c r="C57">
+        <v>8.602693604000001</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B58">
+        <v>2023</v>
+      </c>
+      <c r="C58">
+        <v>8.511753353</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B59">
+        <v>2017</v>
+      </c>
+      <c r="C59">
+        <v>8.335137311</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B60">
+        <v>2022</v>
+      </c>
+      <c r="C60">
+        <v>8.292907229000001</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Textiles/leather</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B61">
+        <v>2021</v>
+      </c>
+      <c r="C61">
+        <v>8.236747536999999</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Textiles/leather</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B62">
+        <v>2019</v>
+      </c>
+      <c r="C62">
+        <v>8.045917774999999</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Plastics/rubber</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B63">
+        <v>2018</v>
+      </c>
+      <c r="C63">
+        <v>7.989860336</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Plastics/rubber</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B64">
+        <v>2017</v>
+      </c>
+      <c r="C64">
+        <v>7.933302637</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Plastics/rubber</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B65">
+        <v>2020</v>
+      </c>
+      <c r="C65">
+        <v>7.916098908</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B66">
+        <v>2020</v>
+      </c>
+      <c r="C66">
+        <v>7.864770901</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Textiles/leather</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B67">
+        <v>2020</v>
+      </c>
+      <c r="C67">
+        <v>7.791818931</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Plastics/rubber</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B68">
+        <v>2024</v>
+      </c>
+      <c r="C68">
+        <v>7.605402191</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Plastics/rubber</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B69">
+        <v>2024</v>
+      </c>
+      <c r="C69">
+        <v>7.519005991</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Textiles/leather</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B70">
+        <v>2022</v>
+      </c>
+      <c r="C70">
+        <v>7.433258927</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Plastics/rubber</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B71">
+        <v>2023</v>
+      </c>
+      <c r="C71">
+        <v>7.410469589</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Plastics/rubber</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B72">
+        <v>2023</v>
+      </c>
+      <c r="C72">
+        <v>7.370225776</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Textiles/leather</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B73">
+        <v>2021</v>
+      </c>
+      <c r="C73">
+        <v>7.086138657999999</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Plastics/rubber</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>05</t>
         </is>
       </c>
-      <c r="B11">
+      <c r="B74">
+        <v>2021</v>
+      </c>
+      <c r="C74">
+        <v>6.323440388</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Meat/seafood</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B75">
+        <v>2022</v>
+      </c>
+      <c r="C75">
+        <v>5.891832195</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Meat/seafood</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B76">
+        <v>2019</v>
+      </c>
+      <c r="C76">
+        <v>5.830540881</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Meat/seafood</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B77">
+        <v>2018</v>
+      </c>
+      <c r="C77">
+        <v>5.797327154</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Meat/seafood</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B78">
+        <v>2017</v>
+      </c>
+      <c r="C78">
         <v>5.676988486</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Meat/seafood</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B79">
+        <v>2024</v>
+      </c>
+      <c r="C79">
+        <v>5.673250976999999</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Meat/seafood</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B80">
+        <v>2023</v>
+      </c>
+      <c r="C80">
+        <v>5.615452031</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Meat/seafood</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B81">
+        <v>2020</v>
+      </c>
+      <c r="C81">
+        <v>5.58520028</v>
+      </c>
+      <c r="D81" t="inlineStr">
         <is>
           <t>Meat/seafood</t>
         </is>

</xml_diff>

<commit_message>
Add current-dollar value alongside constant 2017-dollar value throughout
Pivots current_value_YYYY into the long-format data (backfilled to
value_2017_dollars for the 2017 base year) and mirrors it into every
value-based summary, xlsx export, and chart: Totals, top-10
destinations, top-10 export products (ranking/xlsx/intra breakdown),
mode value + mode value-share, and top-10 imports. Rankings stay based
on constant 2017 dollars for consistency; each chart gets a separate
real-dollar and current-dollar version rather than a dual-axis plot.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/top_ten_imp_val.xlsx
+++ b/data/top_ten_imp_val.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -367,10 +367,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>total_value</t>
+          <t>total_value_2017_dollars</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>total_value_current</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -388,7 +393,10 @@
       <c r="C2">
         <v>22.563254868</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2">
+        <v>22.563254868</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Mixed freight</t>
         </is>
@@ -406,7 +414,10 @@
       <c r="C3">
         <v>22.424935147</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3">
+        <v>22.687385625</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Mixed freight</t>
         </is>
@@ -424,7 +435,10 @@
       <c r="C4">
         <v>22.050052484</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4">
+        <v>22.65214653</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Mixed freight</t>
         </is>
@@ -442,7 +456,10 @@
       <c r="C5">
         <v>21.950277688</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5">
+        <v>25.00534327</v>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Mixed freight</t>
         </is>
@@ -460,7 +477,10 @@
       <c r="C6">
         <v>21.908817899</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6">
+        <v>22.773898421</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>Mixed freight</t>
         </is>
@@ -478,7 +498,10 @@
       <c r="C7">
         <v>21.60464556</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7">
+        <v>28.342498564</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>Mixed freight</t>
         </is>
@@ -496,7 +519,10 @@
       <c r="C8">
         <v>21.550885787</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8">
+        <v>29.082555967</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>Mixed freight</t>
         </is>
@@ -514,7 +540,10 @@
       <c r="C9">
         <v>21.453375756</v>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9">
+        <v>28.717489446</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>Mixed freight</t>
         </is>
@@ -532,7 +561,10 @@
       <c r="C10">
         <v>20.664648327</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10">
+        <v>23.501997631</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
@@ -550,7 +582,10 @@
       <c r="C11">
         <v>20.496012635</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11">
+        <v>21.547281495</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
@@ -568,7 +603,10 @@
       <c r="C12">
         <v>20.212253286</v>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12">
+        <v>23.787997689</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
@@ -586,7 +624,10 @@
       <c r="C13">
         <v>19.82979635</v>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13">
+        <v>19.82979635</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
@@ -604,7 +645,10 @@
       <c r="C14">
         <v>19.800400492</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14">
+        <v>23.834401591</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
@@ -622,7 +666,10 @@
       <c r="C15">
         <v>19.606980378</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15">
+        <v>19.826011119</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
@@ -640,7 +687,10 @@
       <c r="C16">
         <v>18.91087282</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16">
+        <v>19.323486076</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
@@ -658,7 +708,10 @@
       <c r="C17">
         <v>18.863957827</v>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17">
+        <v>19.400865263</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
@@ -676,7 +729,10 @@
       <c r="C18">
         <v>15.336451874</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18">
+        <v>18.529848039</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
@@ -694,7 +750,10 @@
       <c r="C19">
         <v>14.240153149</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19">
+        <v>16.854419931</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
@@ -712,7 +771,10 @@
       <c r="C20">
         <v>14.195971537</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20">
+        <v>16.279963746</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
@@ -730,7 +792,10 @@
       <c r="C21">
         <v>13.22208058</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21">
+        <v>14.258183076</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
@@ -748,7 +813,10 @@
       <c r="C22">
         <v>13.147697112</v>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22">
+        <v>13.147697112</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
@@ -766,7 +834,10 @@
       <c r="C23">
         <v>13.007627208</v>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23">
+        <v>15.293160918</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>Misc. mfg. prods.</t>
         </is>
@@ -784,7 +855,10 @@
       <c r="C24">
         <v>12.925027427</v>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24">
+        <v>13.632344388</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>Misc. mfg. prods.</t>
         </is>
@@ -802,7 +876,10 @@
       <c r="C25">
         <v>12.729998436</v>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25">
+        <v>14.261432928</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
@@ -820,7 +897,10 @@
       <c r="C26">
         <v>12.151812909</v>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26">
+        <v>12.682034479</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
@@ -838,7 +918,10 @@
       <c r="C27">
         <v>12.117560532</v>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27">
+        <v>12.117560532</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>Misc. mfg. prods.</t>
         </is>
@@ -856,7 +939,10 @@
       <c r="C28">
         <v>12.053701458</v>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28">
+        <v>12.215290044</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>Precision instruments</t>
         </is>
@@ -874,7 +960,10 @@
       <c r="C29">
         <v>12.02595023</v>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29">
+        <v>12.783556927</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>Precision instruments</t>
         </is>
@@ -892,7 +981,10 @@
       <c r="C30">
         <v>11.976296982</v>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30">
+        <v>11.976296982</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>Precision instruments</t>
         </is>
@@ -910,7 +1002,10 @@
       <c r="C31">
         <v>11.804498361</v>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31">
+        <v>12.058158132</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>Misc. mfg. prods.</t>
         </is>
@@ -928,7 +1023,10 @@
       <c r="C32">
         <v>11.76864921</v>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32">
+        <v>12.936082452</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
@@ -946,7 +1044,10 @@
       <c r="C33">
         <v>11.7157602</v>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33">
+        <v>11.844658192</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>Motorized vehicles</t>
         </is>
@@ -964,7 +1065,10 @@
       <c r="C34">
         <v>11.708666003</v>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34">
+        <v>12.095771905</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>Precision instruments</t>
         </is>
@@ -982,7 +1086,10 @@
       <c r="C35">
         <v>11.688858687</v>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35">
+        <v>15.34161746</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>Misc. mfg. prods.</t>
         </is>
@@ -1000,7 +1107,10 @@
       <c r="C36">
         <v>11.56394589</v>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36">
+        <v>12.264686881</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>Misc. mfg. prods.</t>
         </is>
@@ -1018,7 +1128,10 @@
       <c r="C37">
         <v>11.492383889</v>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37">
+        <v>11.709288266</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>Motorized vehicles</t>
         </is>
@@ -1036,7 +1149,10 @@
       <c r="C38">
         <v>11.489950168</v>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38">
+        <v>13.427238344</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>Motorized vehicles</t>
         </is>
@@ -1054,7 +1170,10 @@
       <c r="C39">
         <v>11.440443032</v>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39">
+        <v>12.888882684</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>Precision instruments</t>
         </is>
@@ -1072,7 +1191,10 @@
       <c r="C40">
         <v>11.405761791</v>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40">
+        <v>13.192841443</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>Motorized vehicles</t>
         </is>
@@ -1090,7 +1212,10 @@
       <c r="C41">
         <v>11.399923779</v>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41">
+        <v>11.946008791</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>Precision instruments</t>
         </is>
@@ -1108,7 +1233,10 @@
       <c r="C42">
         <v>11.335657705</v>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42">
+        <v>11.335657705</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>Motorized vehicles</t>
         </is>
@@ -1126,7 +1254,10 @@
       <c r="C43">
         <v>11.251168751</v>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43">
+        <v>12.700307139</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>Motorized vehicles</t>
         </is>
@@ -1144,7 +1275,10 @@
       <c r="C44">
         <v>11.015596751</v>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44">
+        <v>13.031170096</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>Precision instruments</t>
         </is>
@@ -1162,7 +1296,10 @@
       <c r="C45">
         <v>10.99514825</v>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45">
+        <v>13.411363749</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>Precision instruments</t>
         </is>
@@ -1180,7 +1317,10 @@
       <c r="C46">
         <v>10.666123471</v>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46">
+        <v>11.266633318</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>Motorized vehicles</t>
         </is>
@@ -1198,7 +1338,10 @@
       <c r="C47">
         <v>10.503970719</v>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47">
+        <v>14.385173539</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>Misc. mfg. prods.</t>
         </is>
@@ -1216,7 +1359,10 @@
       <c r="C48">
         <v>10.111668516</v>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48">
+        <v>10.310111532</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>Motorized vehicles</t>
         </is>
@@ -1234,7 +1380,10 @@
       <c r="C49">
         <v>9.960329438999999</v>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49">
+        <v>14.522608901</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>Misc. mfg. prods.</t>
         </is>
@@ -1252,7 +1401,10 @@
       <c r="C50">
         <v>9.34841215</v>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50">
+        <v>9.34841215</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>Textiles/leather</t>
         </is>
@@ -1270,7 +1422,10 @@
       <c r="C51">
         <v>9.155250655</v>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51">
+        <v>9.421482173000001</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>Textiles/leather</t>
         </is>
@@ -1288,7 +1443,10 @@
       <c r="C52">
         <v>9.094969187999999</v>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52">
+        <v>10.01455205</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>Machinery</t>
         </is>
@@ -1306,7 +1464,10 @@
       <c r="C53">
         <v>9.031668614000001</v>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53">
+        <v>11.080900693</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>Machinery</t>
         </is>
@@ -1324,7 +1485,10 @@
       <c r="C54">
         <v>9.007596475</v>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54">
+        <v>9.205002922</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>Machinery</t>
         </is>
@@ -1342,7 +1506,10 @@
       <c r="C55">
         <v>8.944119272</v>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55">
+        <v>9.392511251</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>Machinery</t>
         </is>
@@ -1360,7 +1527,10 @@
       <c r="C56">
         <v>8.799151495</v>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56">
+        <v>9.171133887</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>Textiles/leather</t>
         </is>
@@ -1378,7 +1548,10 @@
       <c r="C57">
         <v>8.602693604000001</v>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57">
+        <v>11.720121791</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>Machinery</t>
         </is>
@@ -1396,7 +1569,10 @@
       <c r="C58">
         <v>8.511753353</v>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58">
+        <v>11.122072992</v>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>Machinery</t>
         </is>
@@ -1414,7 +1590,10 @@
       <c r="C59">
         <v>8.335137311</v>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59">
+        <v>8.335137311</v>
+      </c>
+      <c r="E59" t="inlineStr">
         <is>
           <t>Machinery</t>
         </is>
@@ -1432,7 +1611,10 @@
       <c r="C60">
         <v>8.292907229000001</v>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60">
+        <v>10.300558174</v>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>Textiles/leather</t>
         </is>
@@ -1450,7 +1632,10 @@
       <c r="C61">
         <v>8.236747536999999</v>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61">
+        <v>9.190542112999999</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>Textiles/leather</t>
         </is>
@@ -1468,7 +1653,10 @@
       <c r="C62">
         <v>8.045917774999999</v>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62">
+        <v>8.187356333</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>Plastics/rubber</t>
         </is>
@@ -1486,7 +1674,10 @@
       <c r="C63">
         <v>7.989860336</v>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63">
+        <v>8.291007921</v>
+      </c>
+      <c r="E63" t="inlineStr">
         <is>
           <t>Plastics/rubber</t>
         </is>
@@ -1504,7 +1695,10 @@
       <c r="C64">
         <v>7.933302637</v>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64">
+        <v>7.933302637</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>Plastics/rubber</t>
         </is>
@@ -1522,7 +1716,10 @@
       <c r="C65">
         <v>7.916098908</v>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65">
+        <v>8.428583952999999</v>
+      </c>
+      <c r="E65" t="inlineStr">
         <is>
           <t>Machinery</t>
         </is>
@@ -1540,7 +1737,10 @@
       <c r="C66">
         <v>7.864770901</v>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66">
+        <v>8.145022535000001</v>
+      </c>
+      <c r="E66" t="inlineStr">
         <is>
           <t>Textiles/leather</t>
         </is>
@@ -1558,7 +1758,10 @@
       <c r="C67">
         <v>7.791818931</v>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D67">
+        <v>7.781526337</v>
+      </c>
+      <c r="E67" t="inlineStr">
         <is>
           <t>Plastics/rubber</t>
         </is>
@@ -1576,7 +1779,10 @@
       <c r="C68">
         <v>7.605402191</v>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D68">
+        <v>9.940455029000001</v>
+      </c>
+      <c r="E68" t="inlineStr">
         <is>
           <t>Plastics/rubber</t>
         </is>
@@ -1594,7 +1800,10 @@
       <c r="C69">
         <v>7.519005991</v>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69">
+        <v>9.443005038999999</v>
+      </c>
+      <c r="E69" t="inlineStr">
         <is>
           <t>Textiles/leather</t>
         </is>
@@ -1612,7 +1821,10 @@
       <c r="C70">
         <v>7.433258927</v>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D70">
+        <v>10.061683294</v>
+      </c>
+      <c r="E70" t="inlineStr">
         <is>
           <t>Plastics/rubber</t>
         </is>
@@ -1630,7 +1842,10 @@
       <c r="C71">
         <v>7.410469589</v>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="D71">
+        <v>9.752391736</v>
+      </c>
+      <c r="E71" t="inlineStr">
         <is>
           <t>Plastics/rubber</t>
         </is>
@@ -1648,7 +1863,10 @@
       <c r="C72">
         <v>7.370225776</v>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D72">
+        <v>9.230021084000001</v>
+      </c>
+      <c r="E72" t="inlineStr">
         <is>
           <t>Textiles/leather</t>
         </is>
@@ -1666,7 +1884,10 @@
       <c r="C73">
         <v>7.086138657999999</v>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D73">
+        <v>8.508362349999999</v>
+      </c>
+      <c r="E73" t="inlineStr">
         <is>
           <t>Plastics/rubber</t>
         </is>
@@ -1684,7 +1905,10 @@
       <c r="C74">
         <v>6.323440388</v>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D74">
+        <v>7.629748324</v>
+      </c>
+      <c r="E74" t="inlineStr">
         <is>
           <t>Meat/seafood</t>
         </is>
@@ -1702,7 +1926,10 @@
       <c r="C75">
         <v>5.891832195</v>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D75">
+        <v>7.471407187</v>
+      </c>
+      <c r="E75" t="inlineStr">
         <is>
           <t>Meat/seafood</t>
         </is>
@@ -1720,7 +1947,10 @@
       <c r="C76">
         <v>5.830540881</v>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D76">
+        <v>5.817995336</v>
+      </c>
+      <c r="E76" t="inlineStr">
         <is>
           <t>Meat/seafood</t>
         </is>
@@ -1738,7 +1968,10 @@
       <c r="C77">
         <v>5.797327154</v>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D77">
+        <v>5.65075676</v>
+      </c>
+      <c r="E77" t="inlineStr">
         <is>
           <t>Meat/seafood</t>
         </is>
@@ -1756,7 +1989,10 @@
       <c r="C78">
         <v>5.676988486</v>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D78">
+        <v>5.676988486</v>
+      </c>
+      <c r="E78" t="inlineStr">
         <is>
           <t>Meat/seafood</t>
         </is>
@@ -1774,7 +2010,10 @@
       <c r="C79">
         <v>5.673250976999999</v>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D79">
+        <v>7.274609227</v>
+      </c>
+      <c r="E79" t="inlineStr">
         <is>
           <t>Meat/seafood</t>
         </is>
@@ -1792,7 +2031,10 @@
       <c r="C80">
         <v>5.615452031</v>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D80">
+        <v>6.924839711</v>
+      </c>
+      <c r="E80" t="inlineStr">
         <is>
           <t>Meat/seafood</t>
         </is>
@@ -1810,7 +2052,10 @@
       <c r="C81">
         <v>5.58520028</v>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D81">
+        <v>5.669323803</v>
+      </c>
+      <c r="E81" t="inlineStr">
         <is>
           <t>Meat/seafood</t>
         </is>

</xml_diff>